<commit_message>
feat(providers): add and update Type of Program options across directory, form modal, and AI import
</commit_message>
<xml_diff>
--- a/AI_Import_Template.xlsx
+++ b/AI_Import_Template.xlsx
@@ -397,21 +397,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N7"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
     <col min="3" max="3" width="20.83203125" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="23.83203125" customWidth="1"/>
-    <col min="6" max="6" width="29.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="31.83203125" customWidth="1"/>
-    <col min="9" max="9" width="22.83203125" customWidth="1"/>
-    <col min="10" max="10" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="23.83203125" customWidth="1"/>
+    <col min="7" max="7" width="29.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="31.83203125" customWidth="1"/>
+    <col min="10" max="10" width="22.83203125" customWidth="1"/>
     <col min="11" max="11" width="20.83203125" customWidth="1"/>
     <col min="12" max="12" width="20.83203125" customWidth="1"/>
-    <col min="13" max="13" width="30.83203125" customWidth="1"/>
+    <col min="13" max="13" width="20.83203125" customWidth="1"/>
+    <col min="14" max="14" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,33 +426,36 @@
         <v>Classification</v>
       </c>
       <c r="D1" t="str">
+        <v>Type of Program</v>
+      </c>
+      <c r="E1" t="str">
         <v>Sector</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Qualification Title</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>Training Duration (Hours)</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>SIL Duration (Hours)</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Program Registration Number</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Date of Expiration</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>School ID</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Complete Address</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Contact Number</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Email / Website / Facebook</v>
       </c>
     </row>
@@ -466,33 +470,36 @@
         <v>SUC</v>
       </c>
       <c r="D2" t="str">
+        <v>IBT</v>
+      </c>
+      <c r="E2" t="str">
         <v>Information and Communication Technology</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>Computer Systems Servicing NC II</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>160</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>40</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>WTR-0920140046</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>12/31/2027</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>SCH-001234</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>673 Quirino Highway, San Bartolome, Novaliches, Quezon City</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>(02) 8806-3049</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>qcpu.edu.ph</v>
       </c>
     </row>
@@ -507,33 +514,36 @@
         <v>TTI</v>
       </c>
       <c r="D3" t="str">
+        <v>Diploma</v>
+      </c>
+      <c r="E3" t="str">
         <v>Electronics</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>Electronics Products Assembly Servicing NC II</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>218</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>60</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>NTR-0820170089</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>06/30/2028</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>SCH-005678</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Brgy. Western Bicutan, Taguig City</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>0917-123-4567</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>tesda-tti-taguig@fb.com</v>
       </c>
     </row>
@@ -548,39 +558,174 @@
         <v>HEI</v>
       </c>
       <c r="D4" t="str">
+        <v>Bundled</v>
+      </c>
+      <c r="E4" t="str">
         <v>Information and Communication Technology</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <v>Bookkeeping NC III</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>292</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>80</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>WTR-1320180034</v>
       </c>
-      <c r="I4" t="str">
+      <c r="J4" t="str">
         <v>03/15/2026</v>
       </c>
-      <c r="J4" t="str">
+      <c r="K4" t="str">
         <v>SCH-009012</v>
       </c>
-      <c r="K4" t="str">
+      <c r="L4" t="str">
         <v>180 EDSA, Grace Park, Caloocan City</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M4" t="str">
         <v>(02) 8363-1234</v>
       </c>
-      <c r="M4" t="str">
+      <c r="N4" t="str">
         <v>caloocan@sti.edu</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Davao Mobile Skills Center</v>
+      </c>
+      <c r="B5" t="str">
+        <v>LGU-RUN</v>
+      </c>
+      <c r="C5" t="str">
+        <v>LUC</v>
+      </c>
+      <c r="D5" t="str">
+        <v>MTP</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Agriculture</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Organic Agriculture Production NC II</v>
+      </c>
+      <c r="G5">
+        <v>120</v>
+      </c>
+      <c r="H5">
+        <v>20</v>
+      </c>
+      <c r="I5" t="str">
+        <v>MTP-2024-0099</v>
+      </c>
+      <c r="J5" t="str">
+        <v>10/15/2027</v>
+      </c>
+      <c r="K5" t="str">
+        <v>SCH-003456</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Door 4, City Hall Annex, Davao City</v>
+      </c>
+      <c r="M5" t="str">
+        <v>0918-987-6543</v>
+      </c>
+      <c r="N5" t="str">
+        <v>dmsc@davaocity.gov.ph</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Mindanao Enterprise Training Hub</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Private</v>
+      </c>
+      <c r="C6" t="str">
+        <v>EBET</v>
+      </c>
+      <c r="D6" t="str">
+        <v>EBET</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Manufacturing</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Shielded Metal Arc Welding NC II</v>
+      </c>
+      <c r="G6">
+        <v>268</v>
+      </c>
+      <c r="H6">
+        <v>60</v>
+      </c>
+      <c r="I6" t="str">
+        <v>EBT-2023-0182</v>
+      </c>
+      <c r="J6" t="str">
+        <v>08/20/2026</v>
+      </c>
+      <c r="K6" t="str">
+        <v>SCH-007890</v>
+      </c>
+      <c r="L6" t="str">
+        <v>KM 9, Lanang, Davao City</v>
+      </c>
+      <c r="M6" t="str">
+        <v>(082) 234-5678</v>
+      </c>
+      <c r="N6" t="str">
+        <v>info@meth-davao.com</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Regional Micro-Credential Academy</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Public</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TTI</v>
+      </c>
+      <c r="D7" t="str">
+        <v>MCC</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Tourism</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Front Office Services NC II</v>
+      </c>
+      <c r="G7">
+        <v>80</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7" t="str">
+        <v>MCC-2025-0012</v>
+      </c>
+      <c r="J7" t="str">
+        <v>11/30/2028</v>
+      </c>
+      <c r="K7" t="str">
+        <v>SCH-004567</v>
+      </c>
+      <c r="L7" t="str">
+        <v>R. Castillo St., Agdao, Davao City</v>
+      </c>
+      <c r="M7" t="str">
+        <v>(082) 221-9988</v>
+      </c>
+      <c r="N7" t="str">
+        <v>mcc.academy@tesda.gov.ph</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>